<commit_message>
docs: incorporar el detalle de horas que entrego Alexis Carnero en agosto 2026
Alexis Carnero entrego su propia planilla de agosto (Horas_Agosto_2026_Alexis_Carnero.xlsx). El script la carga como una entrada mas, junto a la de Gabriel Denis, y antes de escribir verifica que cada dia, inicio, fin y horas coincidan con el anexo ya separado.

- Detalle: las 17 filas de Alexis dejan de estar sin descripcion.
- Nota KLG de Alexis: el horario sigue siendo una reconstruccion de KLG, pero ahora consta que el detalle que entrego coincide con ella.
- Tabla 3 del informe: la linea de 59,0 h sin describir se reemplaza por cinco lineas agrupadas por tema (26,5 + 5,0 + 12,0 + 8,5 + 7,0).
- Tabla 4: la explicacion de alertas dice que el detalle esta incorporado y que coincide con la separacion de horas.

Totales sin cambios: 306,0 h y 5.415,00.
</commit_message>
<xml_diff>
--- a/output/2026-08/Anexo-II-A-Detalle-horas-KLG-2026-08.xlsx
+++ b/output/2026-08/Anexo-II-A-Detalle-horas-KLG-2026-08.xlsx
@@ -2292,7 +2292,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F3" s="35" t="n"/>
+      <c r="F3" s="35" t="inlineStr">
+        <is>
+          <t>Reunión "Revisión de Pendientes de Sprints 8, 9 y 10 para aprobar Hito 2" (1,5 h). Análisis del bug del Certificado de Inscripción Vigente en Test (crea_tramite.aspx / DLL Chequeo_Vigencia, RUT 76000001-9): se descarta problema de código y se acota a datos faltantes del inscrito. Entrega de 6 componentes ASP y 1 script SQL con el fix de FECHAENVIOEXTRANET y Antecedentes. Gestión de acceso al repositorio Azure de la API. Despliegue en desarrollo de la API con los parámetros @ICR_FEC_ENV_EXT y @ICR_NUM_FOL_SOL (Req17).</t>
+        </is>
+      </c>
       <c r="G3" s="36" t="n">
         <v>8</v>
       </c>
@@ -2508,7 +2512,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F8" s="29" t="n"/>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>Reunión "Revisión de Últimos Reparos Pendientes" (1 h). Identificación de la causa raíz del bug de emisión de certificado: faltaba el domicilio de casa matriz en la tabla DIRECCION. Relevamiento con SQL Profiler de los datos obligatorios para emitir el Certificado de Vigencia desde Trámites en Línea. Seguimiento de subespecialidades de socios en consulta por duplicidad y del cálculo de vencimiento en sanciones.</t>
+        </is>
+      </c>
       <c r="G8" s="30" t="n">
         <v>7</v>
       </c>
@@ -2529,7 +2537,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2698,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F12" s="29" t="n"/>
+      <c r="F12" s="29" t="inlineStr">
+        <is>
+          <t>Reunión "Hito 2: Revisión de Observaciones del Sprint" (1 h): sanciones que no graban en Test, duplicidad de RUT con despliegue de especialidades, cálculo de experiencia y error al grabar socio con especialidad asociada. Coordinación de traspasos a Test y seguimiento de las entregas v14 a v16 con el equipo y la contraparte usuaria.</t>
+        </is>
+      </c>
       <c r="G12" s="30" t="n">
         <v>6</v>
       </c>
@@ -2711,7 +2723,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -2960,7 +2972,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F18" s="29" t="n"/>
+      <c r="F18" s="29" t="inlineStr">
+        <is>
+          <t>Reunión "Hito 2 - Traspaso a Producción" (30 min). Inventario de componentes .asp de los Sprints 8, 9 y 10 contrastado contra el repositorio; armado y envío de los listados de componentes y scripts SQL del Hito 2 para traspaso a Producción. Revisión de scripts de parametrización por decreto y de las observaciones del Sprint 11 (HU 36-39).</t>
+        </is>
+      </c>
       <c r="G18" s="30" t="n">
         <v>5.5</v>
       </c>
@@ -2981,7 +2997,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -3186,7 +3202,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F23" s="29" t="n"/>
+      <c r="F23" s="29" t="inlineStr">
+        <is>
+          <t>Reunión "Sprint 11 - Reparos de Usuario" (1 h). BUG-107: diagnóstico de la clasificación errónea del Tipo Art. 6 en el Reporte de Consultores y corrección del criterio DS135, que estaba invertido.</t>
+        </is>
+      </c>
       <c r="G23" s="30" t="n">
         <v>1</v>
       </c>
@@ -3207,7 +3227,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -3324,7 +3344,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F26" s="29" t="n"/>
+      <c r="F26" s="29" t="inlineStr">
+        <is>
+          <t>Dos reuniones: "ERRORES en producción" (1 h) y "PPTT y RRTT - Revisar Sprint 11 y 12" (1 h). Análisis del fallo de los scripts de parametrización por decreto en Producción: dependen de una columna inexistente, por lo que deben ejecutarse antes los scripts de auditoría del Req14. Entrega del fix de mayúsculas en "Profesional Habilitante" del Certificado de Vigencia, en versiones para RRTT y Portal Trámites en Línea. Continuación de BUG-107.</t>
+        </is>
+      </c>
       <c r="G26" s="30" t="n">
         <v>5</v>
       </c>
@@ -3345,7 +3369,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -3594,7 +3618,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F32" s="29" t="n"/>
+      <c r="F32" s="29" t="inlineStr">
+        <is>
+          <t>Reunión "Revisar Sprint 11 Hito 2" (1 h) y daily. Fix del "ERROR EN RT" y verificación en desarrollo. Filtro de antecedentes acotado a Consultores con corte de decreto 2027-01-01, y ajuste posterior para que el "Certificado de Vigencia del Registro de Comercio" aparezca en inscripciones previas al decreto. Validación en Test. Verificación del incidente de documentación de socios en Constructores, Contratistas y Consultores.</t>
+        </is>
+      </c>
       <c r="G32" s="30" t="n">
         <v>6</v>
       </c>
@@ -3615,7 +3643,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3804,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F36" s="29" t="n"/>
+      <c r="F36" s="29" t="inlineStr">
+        <is>
+          <t>Fix de producción sobre atr_modifica_socio.asp.</t>
+        </is>
+      </c>
       <c r="G36" s="30" t="n">
         <v>1</v>
       </c>
@@ -3797,7 +3829,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -4002,7 +4034,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F41" s="29" t="n"/>
+      <c r="F41" s="29" t="inlineStr">
+        <is>
+          <t>Reunión "RRTT - Revisión de Incidencias en Producción" (1 h). Entregav31: BUG-109 (Type mismatch cal_jur), BUG-110 (acentos y caracteres corruptos en el Informe Jurídico), error ASP 0140 por @LANGUAGE duplicado y ajuste de los límites de Fecha de Nacimiento y Constitución.</t>
+        </is>
+      </c>
       <c r="G41" s="30" t="n">
         <v>2</v>
       </c>
@@ -4023,7 +4059,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -4140,7 +4176,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F44" s="29" t="n"/>
+      <c r="F44" s="29" t="inlineStr">
+        <is>
+          <t>Entrega urgente del listado de componentes y scripts del Hito 3 / Sprint 11 para paso a Producción. Diagnóstico y corrección del error de integración PPTT-RRTT en el ingreso de solicitudes de Contratistas: el repositorio Azure de la API estaba desactualizado respecto del binario en servicio. Verificación de que el mismo fix cubre un segundo error reportado. Revisión Entregav27-32 y corrección de 3 corrupciones no reportadas.</t>
+        </is>
+      </c>
       <c r="G44" s="30" t="n">
         <v>6.5</v>
       </c>
@@ -4161,7 +4201,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4362,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F48" s="29" t="n"/>
+      <c r="F48" s="29" t="inlineStr">
+        <is>
+          <t>Recepción y primer análisis del incidente "Error en Informe Jurídico, Rol SEREMI", reportado desde Producción por varias regiones.</t>
+        </is>
+      </c>
       <c r="G48" s="30" t="n">
         <v>1</v>
       </c>
@@ -4406,7 +4450,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F50" s="29" t="n"/>
+      <c r="F50" s="29" t="inlineStr">
+        <is>
+          <t>Reunión "Informo falla en sistema RT" (30 min). BUG-115: diagnóstico del desborde de Integer en el DLL VB6 al modificar informes con ID superior a 32.767, y reemplazo por el SP USP_UPD_INFORME_JURIDICO. Revisión del ETL del Observatorio (Power BI) y del paquete SSIS.</t>
+        </is>
+      </c>
       <c r="G50" s="30" t="n">
         <v>1</v>
       </c>
@@ -4427,7 +4475,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -4544,7 +4592,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F53" s="29" t="n"/>
+      <c r="F53" s="29" t="inlineStr">
+        <is>
+          <t>Atención de un nuevo error reportado en la integración de Proveedores Técnicos. Seguimiento de la Entregav36, que consolida las correcciones previas e incorpora el SP de informes jurídicos.</t>
+        </is>
+      </c>
       <c r="G53" s="30" t="n">
         <v>1</v>
       </c>
@@ -4565,7 +4617,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4959,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F61" s="29" t="n"/>
+      <c r="F61" s="29" t="inlineStr">
+        <is>
+          <t>Seguimiento del incidente de integración PPTT-RRTT: verificación del estado del fix del 14/08 y su paso a Test, confirmación de pruebas exitosas en desarrollo con solicitudes de Consultores y Contratistas, y reenvío del detalle técnico a la contraparte.</t>
+        </is>
+      </c>
       <c r="G61" s="30" t="n">
         <v>1</v>
       </c>
@@ -4928,7 +4984,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5057,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F63" s="29" t="n"/>
+      <c r="F63" s="29" t="inlineStr">
+        <is>
+          <t>Coordinación de la reunión sobre la toma de razón del decreto que modifica el Registro Nacional. Recepción y revisión de un nuevo error en producción sobre mensajes individuales de B2B. Gestión de credenciales de acceso al repositorio Azure.</t>
+        </is>
+      </c>
       <c r="G63" s="30" t="n">
         <v>2.5</v>
       </c>
@@ -5022,7 +5082,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>
@@ -5139,7 +5199,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F66" s="29" t="n"/>
+      <c r="F66" s="29" t="inlineStr">
+        <is>
+          <t>Reunión "Cápsula Jurídica - Toma de razón del decreto que modifica el Registro Nacional" (1 h). API SyncDocumental (GesDoc): resolución del RUT del titular ampliada a equipo de trabajo, nómina de trabajadores y nómina de asesores; reubicación de la validación de tipo de documento; rutas de file server leídas desde configuración.</t>
+        </is>
+      </c>
       <c r="G66" s="30" t="n">
         <v>2.5</v>
       </c>
@@ -5575,7 +5639,11 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F76" s="29" t="n"/>
+      <c r="F76" s="29" t="inlineStr">
+        <is>
+          <t>Reunión "PPTT y RRTT - Revisar precisiones a compromisos" (1 h). Revisión del informe de QA (Aranda 1349249) y del selector Antiguo/Actual D.S. N°135 para los buscadores de inscritos.</t>
+        </is>
+      </c>
       <c r="G76" s="30" t="n">
         <v>2</v>
       </c>
@@ -5596,7 +5664,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: sacar el campo archivo de personas, que ya no se escribe en ningun lado
</commit_message>
<xml_diff>
--- a/output/2026-08/Anexo-II-A-Detalle-horas-KLG-2026-08.xlsx
+++ b/output/2026-08/Anexo-II-A-Detalle-horas-KLG-2026-08.xlsx
@@ -763,12 +763,10 @@
           <t>Horas en Kimai según C.UNIX</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
-        <v>306</v>
-      </c>
+      <c r="B5" s="8" t="n"/>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Registros de Kimai al 29/09/2026. Coinciden día por día con las exportaciones enviadas por KLG.</t>
+          <t>C.UNIX anota aca el total que le da Kimai; la diferencia de abajo debe ser 0.</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1878,7 @@
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>Alexis Carnero</t>
+          <t>Gabriel Denis</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
@@ -1888,11 +1886,7 @@
           <t>Desarrollador</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>acarnero</t>
-        </is>
-      </c>
+      <c r="C8" s="16" t="n"/>
       <c r="E8" s="16" t="inlineStr">
         <is>
           <t>SELICO</t>
@@ -1910,7 +1904,7 @@
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>Franco Dodera</t>
+          <t>Matias Zalazar</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
@@ -1920,7 +1914,7 @@
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>franco</t>
+          <t>mzalazar</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
@@ -1940,7 +1934,7 @@
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>Matias Zalazar</t>
+          <t>Franco Dodera</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
@@ -1950,7 +1944,7 @@
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>mzalazar</t>
+          <t>franco</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
@@ -1970,7 +1964,7 @@
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>Lautaro Zalazar</t>
+          <t>Alexis Carnero</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
@@ -1980,7 +1974,7 @@
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>lzalazar</t>
+          <t>acarnero</t>
         </is>
       </c>
       <c r="E11" s="16" t="inlineStr">
@@ -2000,7 +1994,7 @@
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>Luciano Carducci</t>
+          <t>Lautaro Zalazar</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
@@ -2010,7 +2004,7 @@
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>lcarducci</t>
+          <t>lzalazar</t>
         </is>
       </c>
       <c r="E12" s="16" t="inlineStr">
@@ -2030,7 +2024,7 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Gabriel Denis</t>
+          <t>Luciano Carducci</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
@@ -2038,7 +2032,11 @@
           <t>Desarrollador</t>
         </is>
       </c>
-      <c r="C13" s="16" t="n"/>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>lcarducci</t>
+        </is>
+      </c>
       <c r="E13" s="16" t="n"/>
       <c r="F13" s="16" t="n"/>
       <c r="G13" s="17" t="n"/>
@@ -2227,12 +2225,8 @@
       <c r="A2" s="32" t="n">
         <v>46236</v>
       </c>
-      <c r="B2" s="33" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C2" s="33" t="n">
-        <v>0.4270833333333333</v>
-      </c>
+      <c r="B2" s="33" t="n"/>
+      <c r="C2" s="33" t="n"/>
       <c r="D2" s="34" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -2268,7 +2262,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Dia completo de Gabriel Denis, que no tiene usuario de Kimai. Se conserva el horario del bloque original registrado en la cuenta de Alexis Carnero.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -2276,12 +2270,8 @@
       <c r="A3" s="32" t="n">
         <v>46237</v>
       </c>
-      <c r="B3" s="33" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C3" s="33" t="n">
-        <v>0.6770833333333334</v>
-      </c>
+      <c r="B3" s="33" t="n"/>
+      <c r="C3" s="33" t="n"/>
       <c r="D3" s="34" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -2292,11 +2282,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F3" s="35" t="inlineStr">
-        <is>
-          <t>Reunión "Revisión de Pendientes de Sprints 8, 9 y 10 para aprobar Hito 2" (1,5 h). Análisis del bug del Certificado de Inscripción Vigente en Test (crea_tramite.aspx / DLL Chequeo_Vigencia, RUT 76000001-9): se descarta problema de código y se acota a datos faltantes del inscrito. Entrega de 6 componentes ASP y 1 script SQL con el fix de FECHAENVIOEXTRANET y Antecedentes. Gestión de acceso al repositorio Azure de la API. Despliegue en desarrollo de la API con los parámetros @ICR_FEC_ENV_EXT y @ICR_NUM_FOL_SOL (Req17).</t>
-        </is>
-      </c>
+      <c r="F3" s="35" t="n"/>
       <c r="G3" s="36" t="n">
         <v>8</v>
       </c>
@@ -2364,12 +2350,8 @@
       <c r="A5" s="26" t="n">
         <v>46237</v>
       </c>
-      <c r="B5" s="27" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="C5" s="27" t="n">
-        <v>0.6875</v>
-      </c>
+      <c r="B5" s="27" t="n"/>
+      <c r="C5" s="27" t="n"/>
       <c r="D5" s="28" t="inlineStr">
         <is>
           <t>Lautaro Zalazar</t>
@@ -2380,11 +2362,7 @@
           <t>Victorius 3</t>
         </is>
       </c>
-      <c r="F5" s="29" t="inlineStr">
-        <is>
-          <t>Coordinación nuevo proyecto gobierno de córdoba</t>
-        </is>
-      </c>
+      <c r="F5" s="29" t="n"/>
       <c r="G5" s="30" t="n">
         <v>0.5</v>
       </c>
@@ -2430,7 +2408,7 @@
         </is>
       </c>
       <c r="G6" s="30" t="n">
-        <v>0.5</v>
+        <v>0.499999999999992</v>
       </c>
       <c r="H6" s="20">
         <f>IF(A6="","",TRIM(IF(WEEKDAY(A6,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A6,$D$2:$D$601,D6)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B6&lt;&gt;"",C6&lt;&gt;"",C6&lt;B6),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F6))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F6)),ISERROR(SEARCH("CU-",F6))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E6,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D6,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -2496,12 +2474,8 @@
       <c r="A8" s="26" t="n">
         <v>46238</v>
       </c>
-      <c r="B8" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C8" s="27" t="n">
-        <v>0.6354166666666666</v>
-      </c>
+      <c r="B8" s="27" t="n"/>
+      <c r="C8" s="27" t="n"/>
       <c r="D8" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -2512,11 +2486,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F8" s="29" t="inlineStr">
-        <is>
-          <t>Reunión "Revisión de Últimos Reparos Pendientes" (1 h). Identificación de la causa raíz del bug de emisión de certificado: faltaba el domicilio de casa matriz en la tabla DIRECCION. Relevamiento con SQL Profiler de los datos obligatorios para emitir el Certificado de Vigencia desde Trámites en Línea. Seguimiento de subespecialidades de socios en consulta por duplicidad y del cálculo de vencimiento en sanciones.</t>
-        </is>
-      </c>
+      <c r="F8" s="29" t="n"/>
       <c r="G8" s="30" t="n">
         <v>7</v>
       </c>
@@ -2537,7 +2507,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -2589,12 +2559,8 @@
       <c r="A10" s="26" t="n">
         <v>46238</v>
       </c>
-      <c r="B10" s="27" t="n">
-        <v>0.6354166666666666</v>
-      </c>
-      <c r="C10" s="27" t="n">
-        <v>0.96875</v>
-      </c>
+      <c r="B10" s="27" t="n"/>
+      <c r="C10" s="27" t="n"/>
       <c r="D10" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -2630,7 +2596,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -2682,12 +2648,8 @@
       <c r="A12" s="26" t="n">
         <v>46239</v>
       </c>
-      <c r="B12" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C12" s="27" t="n">
-        <v>0.59375</v>
-      </c>
+      <c r="B12" s="27" t="n"/>
+      <c r="C12" s="27" t="n"/>
       <c r="D12" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -2698,11 +2660,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F12" s="29" t="inlineStr">
-        <is>
-          <t>Reunión "Hito 2: Revisión de Observaciones del Sprint" (1 h): sanciones que no graban en Test, duplicidad de RUT con despliegue de especialidades, cálculo de experiencia y error al grabar socio con especialidad asociada. Coordinación de traspasos a Test y seguimiento de las entregas v14 a v16 con el equipo y la contraparte usuaria.</t>
-        </is>
-      </c>
+      <c r="F12" s="29" t="n"/>
       <c r="G12" s="30" t="n">
         <v>6</v>
       </c>
@@ -2723,7 +2681,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -2775,12 +2733,8 @@
       <c r="A14" s="26" t="n">
         <v>46239</v>
       </c>
-      <c r="B14" s="27" t="n">
-        <v>0.59375</v>
-      </c>
-      <c r="C14" s="27" t="n">
-        <v>0.8854166666666666</v>
-      </c>
+      <c r="B14" s="27" t="n"/>
+      <c r="C14" s="27" t="n"/>
       <c r="D14" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -2816,7 +2770,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2800,7 @@
         </is>
       </c>
       <c r="G15" s="30" t="n">
-        <v>1</v>
+        <v>1.000000000000008</v>
       </c>
       <c r="H15" s="20">
         <f>IF(A15="","",TRIM(IF(WEEKDAY(A15,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A15,$D$2:$D$601,D15)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B15&lt;&gt;"",C15&lt;&gt;"",C15&lt;B15),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F15))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F15)),ISERROR(SEARCH("CU-",F15))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E15,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D15,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -2956,12 +2910,8 @@
       <c r="A18" s="26" t="n">
         <v>46240</v>
       </c>
-      <c r="B18" s="27" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="C18" s="27" t="n">
-        <v>0.5625</v>
-      </c>
+      <c r="B18" s="27" t="n"/>
+      <c r="C18" s="27" t="n"/>
       <c r="D18" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -2972,11 +2922,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F18" s="29" t="inlineStr">
-        <is>
-          <t>Reunión "Hito 2 - Traspaso a Producción" (30 min). Inventario de componentes .asp de los Sprints 8, 9 y 10 contrastado contra el repositorio; armado y envío de los listados de componentes y scripts SQL del Hito 2 para traspaso a Producción. Revisión de scripts de parametrización por decreto y de las observaciones del Sprint 11 (HU 36-39).</t>
-        </is>
-      </c>
+      <c r="F18" s="29" t="n"/>
       <c r="G18" s="30" t="n">
         <v>5.5</v>
       </c>
@@ -2997,7 +2943,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -3049,12 +2995,8 @@
       <c r="A20" s="26" t="n">
         <v>46240</v>
       </c>
-      <c r="B20" s="27" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="C20" s="27" t="n">
-        <v>0.8958333333333334</v>
-      </c>
+      <c r="B20" s="27" t="n"/>
+      <c r="C20" s="27" t="n"/>
       <c r="D20" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -3090,7 +3032,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -3186,12 +3128,8 @@
       <c r="A23" s="26" t="n">
         <v>46241</v>
       </c>
-      <c r="B23" s="27" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="C23" s="27" t="n">
-        <v>0.375</v>
-      </c>
+      <c r="B23" s="27" t="n"/>
+      <c r="C23" s="27" t="n"/>
       <c r="D23" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -3202,11 +3140,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F23" s="29" t="inlineStr">
-        <is>
-          <t>Reunión "Sprint 11 - Reparos de Usuario" (1 h). BUG-107: diagnóstico de la clasificación errónea del Tipo Art. 6 en el Reporte de Consultores y corrección del criterio DS135, que estaba invertido.</t>
-        </is>
-      </c>
+      <c r="F23" s="29" t="n"/>
       <c r="G23" s="30" t="n">
         <v>1</v>
       </c>
@@ -3227,7 +3161,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -3279,12 +3213,8 @@
       <c r="A25" s="26" t="n">
         <v>46241</v>
       </c>
-      <c r="B25" s="27" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="C25" s="27" t="n">
-        <v>0.5416666666666666</v>
-      </c>
+      <c r="B25" s="27" t="n"/>
+      <c r="C25" s="27" t="n"/>
       <c r="D25" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -3320,7 +3250,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -3328,12 +3258,8 @@
       <c r="A26" s="26" t="n">
         <v>46244</v>
       </c>
-      <c r="B26" s="27" t="n">
-        <v>0.3333333333333333</v>
-      </c>
-      <c r="C26" s="27" t="n">
-        <v>0.5416666666666666</v>
-      </c>
+      <c r="B26" s="27" t="n"/>
+      <c r="C26" s="27" t="n"/>
       <c r="D26" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -3344,11 +3270,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F26" s="29" t="inlineStr">
-        <is>
-          <t>Dos reuniones: "ERRORES en producción" (1 h) y "PPTT y RRTT - Revisar Sprint 11 y 12" (1 h). Análisis del fallo de los scripts de parametrización por decreto en Producción: dependen de una columna inexistente, por lo que deben ejecutarse antes los scripts de auditoría del Req14. Entrega del fix de mayúsculas en "Profesional Habilitante" del Certificado de Vigencia, en versiones para RRTT y Portal Trámites en Línea. Continuación de BUG-107.</t>
-        </is>
-      </c>
+      <c r="F26" s="29" t="n"/>
       <c r="G26" s="30" t="n">
         <v>5</v>
       </c>
@@ -3369,7 +3291,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -3421,12 +3343,8 @@
       <c r="A28" s="26" t="n">
         <v>46244</v>
       </c>
-      <c r="B28" s="27" t="n">
-        <v>0.5416666666666666</v>
-      </c>
-      <c r="C28" s="27" t="n">
-        <v>0.875</v>
-      </c>
+      <c r="B28" s="27" t="n"/>
+      <c r="C28" s="27" t="n"/>
       <c r="D28" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -3462,7 +3380,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -3470,12 +3388,8 @@
       <c r="A29" s="26" t="n">
         <v>46244</v>
       </c>
-      <c r="B29" s="27" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="C29" s="27" t="n">
-        <v>0.6875</v>
-      </c>
+      <c r="B29" s="27" t="n"/>
+      <c r="C29" s="27" t="n"/>
       <c r="D29" s="28" t="inlineStr">
         <is>
           <t>Lautaro Zalazar</t>
@@ -3486,11 +3400,7 @@
           <t>Victorius 3</t>
         </is>
       </c>
-      <c r="F29" s="29" t="inlineStr">
-        <is>
-          <t>Relevamiento victorius 1</t>
-        </is>
-      </c>
+      <c r="F29" s="29" t="n"/>
       <c r="G29" s="30" t="n">
         <v>1.5</v>
       </c>
@@ -3580,7 +3490,7 @@
         </is>
       </c>
       <c r="G31" s="30" t="n">
-        <v>2</v>
+        <v>1.999999999999992</v>
       </c>
       <c r="H31" s="20">
         <f>IF(A31="","",TRIM(IF(WEEKDAY(A31,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A31,$D$2:$D$601,D31)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B31&lt;&gt;"",C31&lt;&gt;"",C31&lt;B31),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F31))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F31)),ISERROR(SEARCH("CU-",F31))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E31,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D31,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -3602,12 +3512,8 @@
       <c r="A32" s="26" t="n">
         <v>46245</v>
       </c>
-      <c r="B32" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C32" s="27" t="n">
-        <v>0.59375</v>
-      </c>
+      <c r="B32" s="27" t="n"/>
+      <c r="C32" s="27" t="n"/>
       <c r="D32" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -3618,11 +3524,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F32" s="29" t="inlineStr">
-        <is>
-          <t>Reunión "Revisar Sprint 11 Hito 2" (1 h) y daily. Fix del "ERROR EN RT" y verificación en desarrollo. Filtro de antecedentes acotado a Consultores con corte de decreto 2027-01-01, y ajuste posterior para que el "Certificado de Vigencia del Registro de Comercio" aparezca en inscripciones previas al decreto. Validación en Test. Verificación del incidente de documentación de socios en Constructores, Contratistas y Consultores.</t>
-        </is>
-      </c>
+      <c r="F32" s="29" t="n"/>
       <c r="G32" s="30" t="n">
         <v>6</v>
       </c>
@@ -3643,7 +3545,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -3695,12 +3597,8 @@
       <c r="A34" s="26" t="n">
         <v>46245</v>
       </c>
-      <c r="B34" s="27" t="n">
-        <v>0.59375</v>
-      </c>
-      <c r="C34" s="27" t="n">
-        <v>0.9270833333333334</v>
-      </c>
+      <c r="B34" s="27" t="n"/>
+      <c r="C34" s="27" t="n"/>
       <c r="D34" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -3736,7 +3634,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -3766,7 +3664,7 @@
         </is>
       </c>
       <c r="G35" s="30" t="n">
-        <v>2</v>
+        <v>1.999999999999992</v>
       </c>
       <c r="H35" s="20">
         <f>IF(A35="","",TRIM(IF(WEEKDAY(A35,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A35,$D$2:$D$601,D35)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B35&lt;&gt;"",C35&lt;&gt;"",C35&lt;B35),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F35))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F35)),ISERROR(SEARCH("CU-",F35))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E35,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D35,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -3788,12 +3686,8 @@
       <c r="A36" s="26" t="n">
         <v>46246</v>
       </c>
-      <c r="B36" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C36" s="27" t="n">
-        <v>0.3854166666666667</v>
-      </c>
+      <c r="B36" s="27" t="n"/>
+      <c r="C36" s="27" t="n"/>
       <c r="D36" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -3804,11 +3698,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F36" s="29" t="inlineStr">
-        <is>
-          <t>Fix de producción sobre atr_modifica_socio.asp.</t>
-        </is>
-      </c>
+      <c r="F36" s="29" t="n"/>
       <c r="G36" s="30" t="n">
         <v>1</v>
       </c>
@@ -3829,7 +3719,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -3881,12 +3771,8 @@
       <c r="A38" s="26" t="n">
         <v>46246</v>
       </c>
-      <c r="B38" s="27" t="n">
-        <v>0.3854166666666667</v>
-      </c>
-      <c r="C38" s="27" t="n">
-        <v>0.5520833333333334</v>
-      </c>
+      <c r="B38" s="27" t="n"/>
+      <c r="C38" s="27" t="n"/>
       <c r="D38" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -3922,7 +3808,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -3952,7 +3838,7 @@
         </is>
       </c>
       <c r="G39" s="30" t="n">
-        <v>0.25</v>
+        <v>0.250000000000008</v>
       </c>
       <c r="H39" s="20">
         <f>IF(A39="","",TRIM(IF(WEEKDAY(A39,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A39,$D$2:$D$601,D39)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B39&lt;&gt;"",C39&lt;&gt;"",C39&lt;B39),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F39))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F39)),ISERROR(SEARCH("CU-",F39))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E39,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D39,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -3996,7 +3882,7 @@
         </is>
       </c>
       <c r="G40" s="30" t="n">
-        <v>2</v>
+        <v>1.999999999999992</v>
       </c>
       <c r="H40" s="20">
         <f>IF(A40="","",TRIM(IF(WEEKDAY(A40,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A40,$D$2:$D$601,D40)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B40&lt;&gt;"",C40&lt;&gt;"",C40&lt;B40),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F40))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F40)),ISERROR(SEARCH("CU-",F40))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E40,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D40,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -4018,12 +3904,8 @@
       <c r="A41" s="26" t="n">
         <v>46247</v>
       </c>
-      <c r="B41" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C41" s="27" t="n">
-        <v>0.4270833333333333</v>
-      </c>
+      <c r="B41" s="27" t="n"/>
+      <c r="C41" s="27" t="n"/>
       <c r="D41" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -4034,11 +3916,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F41" s="29" t="inlineStr">
-        <is>
-          <t>Reunión "RRTT - Revisión de Incidencias en Producción" (1 h). Entregav31: BUG-109 (Type mismatch cal_jur), BUG-110 (acentos y caracteres corruptos en el Informe Jurídico), error ASP 0140 por @LANGUAGE duplicado y ajuste de los límites de Fecha de Nacimiento y Constitución.</t>
-        </is>
-      </c>
+      <c r="F41" s="29" t="n"/>
       <c r="G41" s="30" t="n">
         <v>2</v>
       </c>
@@ -4059,7 +3937,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -4111,12 +3989,8 @@
       <c r="A43" s="26" t="n">
         <v>46247</v>
       </c>
-      <c r="B43" s="27" t="n">
-        <v>0.4270833333333333</v>
-      </c>
-      <c r="C43" s="27" t="n">
-        <v>0.7604166666666666</v>
-      </c>
+      <c r="B43" s="27" t="n"/>
+      <c r="C43" s="27" t="n"/>
       <c r="D43" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -4152,7 +4026,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -4160,12 +4034,8 @@
       <c r="A44" s="26" t="n">
         <v>46248</v>
       </c>
-      <c r="B44" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C44" s="27" t="n">
-        <v>0.6145833333333334</v>
-      </c>
+      <c r="B44" s="27" t="n"/>
+      <c r="C44" s="27" t="n"/>
       <c r="D44" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -4176,11 +4046,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F44" s="29" t="inlineStr">
-        <is>
-          <t>Entrega urgente del listado de componentes y scripts del Hito 3 / Sprint 11 para paso a Producción. Diagnóstico y corrección del error de integración PPTT-RRTT en el ingreso de solicitudes de Contratistas: el repositorio Azure de la API estaba desactualizado respecto del binario en servicio. Verificación de que el mismo fix cubre un segundo error reportado. Revisión Entregav27-32 y corrección de 3 corrupciones no reportadas.</t>
-        </is>
-      </c>
+      <c r="F44" s="29" t="n"/>
       <c r="G44" s="30" t="n">
         <v>6.5</v>
       </c>
@@ -4201,7 +4067,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -4253,12 +4119,8 @@
       <c r="A46" s="26" t="n">
         <v>46248</v>
       </c>
-      <c r="B46" s="27" t="n">
-        <v>0.6145833333333334</v>
-      </c>
-      <c r="C46" s="27" t="n">
-        <v>0.8645833333333334</v>
-      </c>
+      <c r="B46" s="27" t="n"/>
+      <c r="C46" s="27" t="n"/>
       <c r="D46" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -4294,7 +4156,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -4324,7 +4186,7 @@
         </is>
       </c>
       <c r="G47" s="30" t="n">
-        <v>1</v>
+        <v>1.000000000000008</v>
       </c>
       <c r="H47" s="20">
         <f>IF(A47="","",TRIM(IF(WEEKDAY(A47,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A47,$D$2:$D$601,D47)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B47&lt;&gt;"",C47&lt;&gt;"",C47&lt;B47),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F47))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F47)),ISERROR(SEARCH("CU-",F47))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E47,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D47,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -4346,12 +4208,8 @@
       <c r="A48" s="26" t="n">
         <v>46251</v>
       </c>
-      <c r="B48" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C48" s="27" t="n">
-        <v>0.3854166666666667</v>
-      </c>
+      <c r="B48" s="27" t="n"/>
+      <c r="C48" s="27" t="n"/>
       <c r="D48" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -4362,11 +4220,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F48" s="29" t="inlineStr">
-        <is>
-          <t>Recepción y primer análisis del incidente "Error en Informe Jurídico, Rol SEREMI", reportado desde Producción por varias regiones.</t>
-        </is>
-      </c>
+      <c r="F48" s="29" t="n"/>
       <c r="G48" s="30" t="n">
         <v>1</v>
       </c>
@@ -4412,7 +4266,7 @@
         </is>
       </c>
       <c r="G49" s="30" t="n">
-        <v>2</v>
+        <v>1.999999999999992</v>
       </c>
       <c r="H49" s="20">
         <f>IF(A49="","",TRIM(IF(WEEKDAY(A49,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A49,$D$2:$D$601,D49)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B49&lt;&gt;"",C49&lt;&gt;"",C49&lt;B49),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F49))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F49)),ISERROR(SEARCH("CU-",F49))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E49,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D49,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -4434,12 +4288,8 @@
       <c r="A50" s="26" t="n">
         <v>46252</v>
       </c>
-      <c r="B50" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C50" s="27" t="n">
-        <v>0.3854166666666667</v>
-      </c>
+      <c r="B50" s="27" t="n"/>
+      <c r="C50" s="27" t="n"/>
       <c r="D50" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -4450,11 +4300,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F50" s="29" t="inlineStr">
-        <is>
-          <t>Reunión "Informo falla en sistema RT" (30 min). BUG-115: diagnóstico del desborde de Integer en el DLL VB6 al modificar informes con ID superior a 32.767, y reemplazo por el SP USP_UPD_INFORME_JURIDICO. Revisión del ETL del Observatorio (Power BI) y del paquete SSIS.</t>
-        </is>
-      </c>
+      <c r="F50" s="29" t="n"/>
       <c r="G50" s="30" t="n">
         <v>1</v>
       </c>
@@ -4475,7 +4321,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -4527,12 +4373,8 @@
       <c r="A52" s="26" t="n">
         <v>46252</v>
       </c>
-      <c r="B52" s="27" t="n">
-        <v>0.3854166666666667</v>
-      </c>
-      <c r="C52" s="27" t="n">
-        <v>0.5520833333333334</v>
-      </c>
+      <c r="B52" s="27" t="n"/>
+      <c r="C52" s="27" t="n"/>
       <c r="D52" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -4568,7 +4410,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -4576,12 +4418,8 @@
       <c r="A53" s="26" t="n">
         <v>46253</v>
       </c>
-      <c r="B53" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C53" s="27" t="n">
-        <v>0.3854166666666667</v>
-      </c>
+      <c r="B53" s="27" t="n"/>
+      <c r="C53" s="27" t="n"/>
       <c r="D53" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -4592,11 +4430,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F53" s="29" t="inlineStr">
-        <is>
-          <t>Atención de un nuevo error reportado en la integración de Proveedores Técnicos. Seguimiento de la Entregav36, que consolida las correcciones previas e incorpora el SP de informes jurídicos.</t>
-        </is>
-      </c>
+      <c r="F53" s="29" t="n"/>
       <c r="G53" s="30" t="n">
         <v>1</v>
       </c>
@@ -4617,7 +4451,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -4669,12 +4503,8 @@
       <c r="A55" s="26" t="n">
         <v>46253</v>
       </c>
-      <c r="B55" s="27" t="n">
-        <v>0.3854166666666667</v>
-      </c>
-      <c r="C55" s="27" t="n">
-        <v>0.71875</v>
-      </c>
+      <c r="B55" s="27" t="n"/>
+      <c r="C55" s="27" t="n"/>
       <c r="D55" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -4710,7 +4540,7 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -4740,7 +4570,7 @@
         </is>
       </c>
       <c r="G56" s="30" t="n">
-        <v>0.5</v>
+        <v>0.499999999999992</v>
       </c>
       <c r="H56" s="20">
         <f>IF(A56="","",TRIM(IF(WEEKDAY(A56,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A56,$D$2:$D$601,D56)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B56&lt;&gt;"",C56&lt;&gt;"",C56&lt;B56),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F56))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F56)),ISERROR(SEARCH("CU-",F56))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E56,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D56,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -4784,7 +4614,7 @@
         </is>
       </c>
       <c r="G57" s="30" t="n">
-        <v>2</v>
+        <v>1.999999999999992</v>
       </c>
       <c r="H57" s="20">
         <f>IF(A57="","",TRIM(IF(WEEKDAY(A57,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A57,$D$2:$D$601,D57)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B57&lt;&gt;"",C57&lt;&gt;"",C57&lt;B57),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F57))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F57)),ISERROR(SEARCH("CU-",F57))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E57,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D57,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -4806,12 +4636,8 @@
       <c r="A58" s="26" t="n">
         <v>46254</v>
       </c>
-      <c r="B58" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C58" s="27" t="n">
-        <v>0.71875</v>
-      </c>
+      <c r="B58" s="27" t="n"/>
+      <c r="C58" s="27" t="n"/>
       <c r="D58" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -4847,7 +4673,7 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>Dia completo de Gabriel Denis, que no tiene usuario de Kimai. Se conserva el horario del bloque original registrado en la cuenta de Alexis Carnero.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -4877,7 +4703,7 @@
         </is>
       </c>
       <c r="G59" s="30" t="n">
-        <v>4</v>
+        <v>4.00000000000008</v>
       </c>
       <c r="H59" s="20">
         <f>IF(A59="","",TRIM(IF(WEEKDAY(A59,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A59,$D$2:$D$601,D59)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B59&lt;&gt;"",C59&lt;&gt;"",C59&lt;B59),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F59))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F59)),ISERROR(SEARCH("CU-",F59))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E59,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D59,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -4943,12 +4769,8 @@
       <c r="A61" s="26" t="n">
         <v>46258</v>
       </c>
-      <c r="B61" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C61" s="27" t="n">
-        <v>0.3854166666666667</v>
-      </c>
+      <c r="B61" s="27" t="n"/>
+      <c r="C61" s="27" t="n"/>
       <c r="D61" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -4959,11 +4781,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F61" s="29" t="inlineStr">
-        <is>
-          <t>Seguimiento del incidente de integración PPTT-RRTT: verificación del estado del fix del 14/08 y su paso a Test, confirmación de pruebas exitosas en desarrollo con solicitudes de Consultores y Contratistas, y reenvío del detalle técnico a la contraparte.</t>
-        </is>
-      </c>
+      <c r="F61" s="29" t="n"/>
       <c r="G61" s="30" t="n">
         <v>1</v>
       </c>
@@ -4984,7 +4802,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -4992,12 +4810,8 @@
       <c r="A62" s="26" t="n">
         <v>46258</v>
       </c>
-      <c r="B62" s="27" t="n">
-        <v>0.3854166666666667</v>
-      </c>
-      <c r="C62" s="27" t="n">
-        <v>0.4270833333333333</v>
-      </c>
+      <c r="B62" s="27" t="n"/>
+      <c r="C62" s="27" t="n"/>
       <c r="D62" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -5033,7 +4847,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -5041,12 +4855,8 @@
       <c r="A63" s="26" t="n">
         <v>46259</v>
       </c>
-      <c r="B63" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C63" s="27" t="n">
-        <v>0.4479166666666667</v>
-      </c>
+      <c r="B63" s="27" t="n"/>
+      <c r="C63" s="27" t="n"/>
       <c r="D63" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -5057,11 +4867,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F63" s="29" t="inlineStr">
-        <is>
-          <t>Coordinación de la reunión sobre la toma de razón del decreto que modifica el Registro Nacional. Recepción y revisión de un nuevo error en producción sobre mensajes individuales de B2B. Gestión de credenciales de acceso al repositorio Azure.</t>
-        </is>
-      </c>
+      <c r="F63" s="29" t="n"/>
       <c r="G63" s="30" t="n">
         <v>2.5</v>
       </c>
@@ -5082,7 +4888,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -5090,12 +4896,8 @@
       <c r="A64" s="26" t="n">
         <v>46259</v>
       </c>
-      <c r="B64" s="27" t="n">
-        <v>0.4479166666666667</v>
-      </c>
-      <c r="C64" s="27" t="n">
-        <v>0.53125</v>
-      </c>
+      <c r="B64" s="27" t="n"/>
+      <c r="C64" s="27" t="n"/>
       <c r="D64" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -5131,7 +4933,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -5161,7 +4963,7 @@
         </is>
       </c>
       <c r="G65" s="30" t="n">
-        <v>1</v>
+        <v>1.000000000000008</v>
       </c>
       <c r="H65" s="20">
         <f>IF(A65="","",TRIM(IF(WEEKDAY(A65,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A65,$D$2:$D$601,D65)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B65&lt;&gt;"",C65&lt;&gt;"",C65&lt;B65),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F65))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F65)),ISERROR(SEARCH("CU-",F65))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E65,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D65,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -5183,12 +4985,8 @@
       <c r="A66" s="26" t="n">
         <v>46260</v>
       </c>
-      <c r="B66" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C66" s="27" t="n">
-        <v>0.4479166666666667</v>
-      </c>
+      <c r="B66" s="27" t="n"/>
+      <c r="C66" s="27" t="n"/>
       <c r="D66" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -5199,11 +4997,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F66" s="29" t="inlineStr">
-        <is>
-          <t>Reunión "Cápsula Jurídica - Toma de razón del decreto que modifica el Registro Nacional" (1 h). API SyncDocumental (GesDoc): resolución del RUT del titular ampliada a equipo de trabajo, nómina de trabajadores y nómina de asesores; reubicación de la validación de tipo de documento; rutas de file server leídas desde configuración.</t>
-        </is>
-      </c>
+      <c r="F66" s="29" t="n"/>
       <c r="G66" s="30" t="n">
         <v>2.5</v>
       </c>
@@ -5271,12 +5065,8 @@
       <c r="A68" s="26" t="n">
         <v>46260</v>
       </c>
-      <c r="B68" s="27" t="n">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="C68" s="27" t="n">
-        <v>0.75</v>
-      </c>
+      <c r="B68" s="27" t="n"/>
+      <c r="C68" s="27" t="n"/>
       <c r="D68" s="28" t="inlineStr">
         <is>
           <t>Lautaro Zalazar</t>
@@ -5287,11 +5077,7 @@
           <t>Victorius 3</t>
         </is>
       </c>
-      <c r="F68" s="29" t="inlineStr">
-        <is>
-          <t>Análisis funcional para cliente Gobierno de Córdoba</t>
-        </is>
-      </c>
+      <c r="F68" s="29" t="n"/>
       <c r="G68" s="30" t="n">
         <v>4</v>
       </c>
@@ -5337,7 +5123,7 @@
         </is>
       </c>
       <c r="G69" s="30" t="n">
-        <v>0.25</v>
+        <v>0.250000000000008</v>
       </c>
       <c r="H69" s="20">
         <f>IF(A69="","",TRIM(IF(WEEKDAY(A69,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A69,$D$2:$D$601,D69)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B69&lt;&gt;"",C69&lt;&gt;"",C69&lt;B69),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F69))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F69)),ISERROR(SEARCH("CU-",F69))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E69,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D69,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -5381,7 +5167,7 @@
         </is>
       </c>
       <c r="G70" s="30" t="n">
-        <v>2</v>
+        <v>1.999999999999992</v>
       </c>
       <c r="H70" s="20">
         <f>IF(A70="","",TRIM(IF(WEEKDAY(A70,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A70,$D$2:$D$601,D70)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B70&lt;&gt;"",C70&lt;&gt;"",C70&lt;B70),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F70))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F70)),ISERROR(SEARCH("CU-",F70))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E70,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D70,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -5469,7 +5255,7 @@
         </is>
       </c>
       <c r="G72" s="30" t="n">
-        <v>2.5</v>
+        <v>2.50000000000008</v>
       </c>
       <c r="H72" s="20">
         <f>IF(A72="","",TRIM(IF(WEEKDAY(A72,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A72,$D$2:$D$601,D72)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B72&lt;&gt;"",C72&lt;&gt;"",C72&lt;B72),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F72))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F72)),ISERROR(SEARCH("CU-",F72))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E72,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D72,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -5557,7 +5343,7 @@
         </is>
       </c>
       <c r="G74" s="30" t="n">
-        <v>0.5</v>
+        <v>0.499999999999992</v>
       </c>
       <c r="H74" s="20">
         <f>IF(A74="","",TRIM(IF(WEEKDAY(A74,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A74,$D$2:$D$601,D74)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B74&lt;&gt;"",C74&lt;&gt;"",C74&lt;B74),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F74))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F74)),ISERROR(SEARCH("CU-",F74))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E74,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D74,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -5601,7 +5387,7 @@
         </is>
       </c>
       <c r="G75" s="30" t="n">
-        <v>3.5</v>
+        <v>3.49999999999992</v>
       </c>
       <c r="H75" s="20">
         <f>IF(A75="","",TRIM(IF(WEEKDAY(A75,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A75,$D$2:$D$601,D75)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B75&lt;&gt;"",C75&lt;&gt;"",C75&lt;B75),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F75))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F75)),ISERROR(SEARCH("CU-",F75))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E75,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D75,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -5623,12 +5409,8 @@
       <c r="A76" s="26" t="n">
         <v>46262</v>
       </c>
-      <c r="B76" s="27" t="n">
-        <v>0.34375</v>
-      </c>
-      <c r="C76" s="27" t="n">
-        <v>0.4270833333333333</v>
-      </c>
+      <c r="B76" s="27" t="n"/>
+      <c r="C76" s="27" t="n"/>
       <c r="D76" s="28" t="inlineStr">
         <is>
           <t>Alexis Carnero</t>
@@ -5639,11 +5421,7 @@
           <t>SELICO</t>
         </is>
       </c>
-      <c r="F76" s="29" t="inlineStr">
-        <is>
-          <t>Reunión "PPTT y RRTT - Revisar precisiones a compromisos" (1 h). Revisión del informe de QA (Aranda 1349249) y del selector Antiguo/Actual D.S. N°135 para los buscadores de inscritos.</t>
-        </is>
-      </c>
+      <c r="F76" s="29" t="n"/>
       <c r="G76" s="30" t="n">
         <v>2</v>
       </c>
@@ -5664,7 +5442,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG al separar las horas de Gabriel Denis del unico bloque diario que Kimai registro en la cuenta de Alexis Carnero. Alexis Carnero entrego despues su propio detalle de agosto y coincide con esa reconstruccion: mismo dia, mismo inicio, mismo fin y las mismas horas. De ahi sale la descripcion de esta fila.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -5716,12 +5494,8 @@
       <c r="A78" s="26" t="n">
         <v>46262</v>
       </c>
-      <c r="B78" s="27" t="n">
-        <v>0.4270833333333333</v>
-      </c>
-      <c r="C78" s="27" t="n">
-        <v>0.59375</v>
-      </c>
+      <c r="B78" s="27" t="n"/>
+      <c r="C78" s="27" t="n"/>
       <c r="D78" s="28" t="inlineStr">
         <is>
           <t>Gabriel Denis</t>
@@ -5757,7 +5531,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>Horario reconstruido por KLG: Kimai registro un unico bloque diario en la cuenta de Alexis Carnero. El bloque se partio por horario entre Alexis Carnero (principio) y Gabriel Denis (final). Las horas estan respaldadas; el corte dentro del dia es una reconstruccion, no un registro.</t>
+          <t>Horas de Gabriel Denis, que no tiene usuario de Kimai: quedaron cargadas en la cuenta de Alexis Carnero y KLG las separó día por día a partir de la planilla gabriel-denis.xlsx. Las horas de cada uno están respaldadas; el corte dentro del día es una reconstrucción.</t>
         </is>
       </c>
     </row>
@@ -5787,7 +5561,7 @@
         </is>
       </c>
       <c r="G79" s="30" t="n">
-        <v>2.5</v>
+        <v>2.50000000000008</v>
       </c>
       <c r="H79" s="20">
         <f>IF(A79="","",TRIM(IF(WEEKDAY(A79,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A79,$D$2:$D$601,D79)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B79&lt;&gt;"",C79&lt;&gt;"",C79&lt;B79),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F79))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F79)),ISERROR(SEARCH("CU-",F79))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E79,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D79,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -5875,7 +5649,7 @@
         </is>
       </c>
       <c r="G81" s="30" t="n">
-        <v>3.5</v>
+        <v>3.49999999999992</v>
       </c>
       <c r="H81" s="20">
         <f>IF(A81="","",TRIM(IF(WEEKDAY(A81,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A81,$D$2:$D$601,D81)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B81&lt;&gt;"",C81&lt;&gt;"",C81&lt;B81),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F81))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F81)),ISERROR(SEARCH("CU-",F81))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E81,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D81,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -5941,12 +5715,8 @@
       <c r="A83" s="26" t="n">
         <v>46265</v>
       </c>
-      <c r="B83" s="27" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C83" s="27" t="n">
-        <v>0.625</v>
-      </c>
+      <c r="B83" s="27" t="n"/>
+      <c r="C83" s="27" t="n"/>
       <c r="D83" s="28" t="inlineStr">
         <is>
           <t>Lautaro Zalazar</t>
@@ -5957,11 +5727,7 @@
           <t>Victorius 3</t>
         </is>
       </c>
-      <c r="F83" s="29" t="inlineStr">
-        <is>
-          <t>Ampliación estimación gobierno de córdoba</t>
-        </is>
-      </c>
+      <c r="F83" s="29" t="n"/>
       <c r="G83" s="30" t="n">
         <v>3</v>
       </c>
@@ -6007,7 +5773,7 @@
         </is>
       </c>
       <c r="G84" s="30" t="n">
-        <v>1</v>
+        <v>1.000000000000008</v>
       </c>
       <c r="H84" s="20">
         <f>IF(A84="","",TRIM(IF(WEEKDAY(A84,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A84,$D$2:$D$601,D84)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B84&lt;&gt;"",C84&lt;&gt;"",C84&lt;B84),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F84))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F84)),ISERROR(SEARCH("CU-",F84))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E84,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D84,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>
@@ -6051,7 +5817,7 @@
         </is>
       </c>
       <c r="G85" s="30" t="n">
-        <v>1</v>
+        <v>1.000000000000008</v>
       </c>
       <c r="H85" s="20">
         <f>IF(A85="","",TRIM(IF(WEEKDAY(A85,2)&gt;5,"Fin de semana. ","")&amp;IF(SUMIFS($G$2:$G$601,$A$2:$A$601,A85,$D$2:$D$601,D85)&gt;9,"Más de 9 h en el día. ","")&amp;IF(AND(B85&lt;&gt;"",C85&lt;&gt;"",C85&lt;B85),"Cruza la medianoche. ","")&amp;IF(LEN(TRIM(F85))&lt;15,"Sin descripción suficiente. ","")&amp;IF(AND(ISERROR(SEARCH("R-0",F85)),ISERROR(SEARCH("CU-",F85))),"Sin ticket. ","")&amp;IF(ISNA(MATCH(E85,Datos!$E$8:$E$22,0)),"Proyecto sin valor hora. ","")&amp;IF(ISNA(MATCH(D85,Datos!$A$8:$A$22,0)),"Persona fuera del equipo. ","")))</f>

</xml_diff>